<commit_message>
TMTT0012454 TMTT0020659 changes Apr 26 2024
</commit_message>
<xml_diff>
--- a/TestData/LV_TC1197andTC1198AddOpportunityInOpportunityHome.xlsx
+++ b/TestData/LV_TC1197andTC1198AddOpportunityInOpportunityHome.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AFF340-C35A-402C-AC7B-9BB81CE92D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BB60DAF-0BD3-4BCE-9C48-2BEBE2B276F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22200" yWindow="1092" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,6 @@
     <t>StdUser</t>
   </si>
   <si>
-    <t>CaoUser</t>
-  </si>
-  <si>
-    <t>SFCAO User</t>
-  </si>
-  <si>
     <t>Advisory</t>
   </si>
   <si>
@@ -108,6 +102,12 @@
   </si>
   <si>
     <t>Opportunities</t>
+  </si>
+  <si>
+    <t>CF Financial User</t>
+  </si>
+  <si>
+    <t>Profile</t>
   </si>
 </sst>
 </file>
@@ -446,15 +446,15 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -473,12 +473,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -496,12 +496,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -519,547 +519,547 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1075,12 +1075,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>